<commit_message>
xls: update template for revenue changes
</commit_message>
<xml_diff>
--- a/config/template.xlsx
+++ b/config/template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\CLionProjects\FinDashCpp\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://islandhousekeywest-my.sharepoint.com/personal/chris_hanagan_islandhousekeywest_com/Documents/FinDash/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5393D4E-397A-4743-B8C4-2169AF7CCB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{B5393D4E-397A-4743-B8C4-2169AF7CCB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{818A3AAB-6F01-4538-9DF2-F4753F1AE7DD}"/>
   <bookViews>
-    <workbookView xWindow="670" yWindow="1460" windowWidth="17060" windowHeight="17050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18940" yWindow="6220" windowWidth="18600" windowHeight="14470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Report" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="53">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -162,9 +162,6 @@
     <t xml:space="preserve">     Guest Privilege</t>
   </si>
   <si>
-    <t xml:space="preserve">     Laundry</t>
-  </si>
-  <si>
     <t xml:space="preserve">     Misc Adjust</t>
   </si>
   <si>
@@ -201,7 +198,7 @@
     <t xml:space="preserve">     Massage</t>
   </si>
   <si>
-    <t xml:space="preserve">     Guest Relations Exp</t>
+    <t xml:space="preserve">     Guest Priv Monthly Min</t>
   </si>
 </sst>
 </file>
@@ -867,7 +864,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1046,10 +1043,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="5" fontId="7" fillId="0" borderId="27" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1100,10 +1093,6 @@
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="40" fontId="18" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -1123,10 +1112,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
@@ -1188,6 +1173,25 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="40" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="40" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="40" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="40" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="40" fontId="7" fillId="0" borderId="27" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="169" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1627,164 +1631,136 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="102">
+      <c r="A3" s="104">
         <v>46165</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
+      <c r="B3" s="104"/>
+      <c r="C3" s="104"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
     </row>
     <row r="4" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="108" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="109"/>
+      <c r="A4" s="110" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="111"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="103" t="s">
+      <c r="D4" s="105" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="104"/>
-      <c r="F4" s="105"/>
+      <c r="E4" s="106"/>
+      <c r="F4" s="107"/>
     </row>
     <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="98"/>
-      <c r="B5" s="99"/>
+      <c r="A5" s="95"/>
+      <c r="B5" s="96"/>
       <c r="C5" s="48"/>
-      <c r="D5" s="106"/>
-      <c r="E5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="109"/>
       <c r="F5" s="50"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="98" t="s">
+      <c r="A6" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="99">
-        <v>9839</v>
-      </c>
+      <c r="B6" s="102"/>
       <c r="C6" s="49"/>
-      <c r="D6" s="106" t="s">
+      <c r="D6" s="108" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="107"/>
-      <c r="F6" s="96">
-        <v>19534.46</v>
-      </c>
+      <c r="E6" s="109"/>
+      <c r="F6" s="93"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="98" t="s">
+      <c r="A7" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="99">
-        <v>24093</v>
-      </c>
-      <c r="C7" s="49">
+      <c r="B7" s="102"/>
+      <c r="C7" s="49" t="e">
         <f>(B6-B7)/B7</f>
-        <v>-0.59162412318930813</v>
-      </c>
-      <c r="D7" s="106" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D7" s="108" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="107"/>
-      <c r="F7" s="96">
-        <f>53154.84+28781.69+24810.66+22467+22045+34218+35912+33240.15+25840.88+19534.46</f>
-        <v>300004.68</v>
-      </c>
+      <c r="E7" s="109"/>
+      <c r="F7" s="93"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="98" t="s">
+      <c r="A8" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="99">
-        <v>200825</v>
-      </c>
+      <c r="B8" s="102"/>
       <c r="C8" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="106" t="s">
+      <c r="D8" s="108" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="107"/>
-      <c r="F8" s="96">
-        <f>145211.69+28268.67</f>
-        <v>173480.36</v>
-      </c>
+      <c r="E8" s="109"/>
+      <c r="F8" s="93"/>
       <c r="G8" s="1"/>
       <c r="I8" s="9"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="98" t="s">
+      <c r="A9" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="99">
-        <v>211219</v>
-      </c>
-      <c r="C9" s="49">
+      <c r="B9" s="102"/>
+      <c r="C9" s="49" t="e">
         <f>(B8-B9)/B9</f>
-        <v>-4.9209588152580967E-2</v>
-      </c>
-      <c r="D9" s="106" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D9" s="108" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="107"/>
-      <c r="F9" s="97">
-        <f>356172.15+19534.46</f>
-        <v>375706.61000000004</v>
-      </c>
+      <c r="E9" s="109"/>
+      <c r="F9" s="94"/>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="100" t="s">
+      <c r="A10" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="99">
-        <v>2645520.4300000002</v>
-      </c>
+      <c r="B10" s="102"/>
       <c r="C10" s="49"/>
-      <c r="D10" s="106"/>
-      <c r="E10" s="107"/>
+      <c r="D10" s="108"/>
+      <c r="E10" s="109"/>
       <c r="F10" s="51"/>
       <c r="G10" s="1"/>
       <c r="H10" s="9"/>
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:9" ht="13" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="101" t="s">
+      <c r="A11" s="98" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="59">
-        <v>2729986</v>
-      </c>
-      <c r="C11" s="49">
+      <c r="B11" s="103"/>
+      <c r="C11" s="49" t="e">
         <f>(B10-B11)/B11</f>
-        <v>-3.0939927897066077E-2</v>
-      </c>
-      <c r="D11" s="106" t="s">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D11" s="108" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="107"/>
-      <c r="F11" s="52">
-        <f>158801.14+75000</f>
-        <v>233801.14</v>
-      </c>
+      <c r="E11" s="109"/>
+      <c r="F11" s="52"/>
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="22"/>
       <c r="B12" s="42"/>
       <c r="C12" s="43"/>
-      <c r="D12" s="106" t="s">
+      <c r="D12" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="107"/>
-      <c r="F12" s="52">
-        <v>-578144.55000000005</v>
-      </c>
+      <c r="E12" s="109"/>
+      <c r="F12" s="52"/>
       <c r="I12" s="1"/>
     </row>
     <row r="13" spans="1:9" ht="13" thickBot="1" x14ac:dyDescent="0.3">
@@ -1795,91 +1771,70 @@
         <v>15</v>
       </c>
       <c r="E13" s="54"/>
-      <c r="F13" s="55">
-        <v>10741.72</v>
-      </c>
+      <c r="F13" s="55"/>
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9" ht="18" x14ac:dyDescent="0.4">
-      <c r="A14" s="103" t="s">
+      <c r="A14" s="105" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="105"/>
+      <c r="B14" s="107"/>
       <c r="C14" s="24"/>
-      <c r="D14" s="103" t="s">
+      <c r="D14" s="105" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="104"/>
-      <c r="F14" s="105"/>
+      <c r="E14" s="106"/>
+      <c r="F14" s="107"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="57" t="s">
-        <v>49</v>
-      </c>
-      <c r="B15" s="85">
-        <v>14095</v>
-      </c>
-      <c r="C15" s="60"/>
-      <c r="D15" s="106" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="82"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="108" t="s">
         <v>18</v>
       </c>
-      <c r="E15" s="107"/>
-      <c r="F15" s="46">
-        <v>14</v>
-      </c>
+      <c r="E15" s="109"/>
+      <c r="F15" s="46"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="86">
-        <v>31</v>
-      </c>
-      <c r="C16" s="60" t="s">
+      <c r="B16" s="83"/>
+      <c r="C16" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="D16" s="106" t="s">
+      <c r="D16" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="107"/>
-      <c r="F16" s="46">
-        <v>13</v>
-      </c>
+      <c r="E16" s="109"/>
+      <c r="F16" s="46"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="62">
-        <f>B15/B16</f>
-        <v>454.67741935483872</v>
-      </c>
+      <c r="B17" s="61"/>
       <c r="C17" s="44"/>
-      <c r="D17" s="106" t="s">
+      <c r="D17" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="107"/>
-      <c r="F17" s="84">
-        <v>602.49</v>
-      </c>
+      <c r="E17" s="109"/>
+      <c r="F17" s="81"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="61">
-        <f>C27/353</f>
-        <v>0</v>
-      </c>
+      <c r="B18" s="60"/>
       <c r="C18" s="44"/>
-      <c r="D18" s="106" t="s">
+      <c r="D18" s="108" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="107"/>
-      <c r="F18" s="63">
-        <f>11538+2432.49+440+602.49</f>
-        <v>15012.98</v>
-      </c>
+      <c r="E18" s="109"/>
+      <c r="F18" s="62"/>
       <c r="G18" s="13"/>
       <c r="H18" t="s">
         <v>0</v>
@@ -1889,30 +1844,22 @@
       <c r="A19" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="61">
-        <f>D27/376</f>
-        <v>0</v>
-      </c>
+      <c r="B19" s="60"/>
       <c r="C19" s="45">
         <f>(B18-B19)</f>
         <v>0</v>
       </c>
-      <c r="D19" s="110" t="s">
+      <c r="D19" s="112" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="111"/>
-      <c r="F19" s="47">
-        <v>0.217</v>
-      </c>
+      <c r="E19" s="113"/>
+      <c r="F19" s="47"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="62">
-        <f>B27/39</f>
-        <v>0</v>
-      </c>
+      <c r="B20" s="61"/>
       <c r="C20" s="25" t="s">
         <v>0</v>
       </c>
@@ -1926,9 +1873,7 @@
       <c r="A21" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="62">
-        <v>0</v>
-      </c>
+      <c r="B21" s="61"/>
       <c r="C21" s="25"/>
       <c r="D21" s="27"/>
       <c r="E21" s="26"/>
@@ -1940,9 +1885,7 @@
       <c r="A22" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="87">
-        <v>0</v>
-      </c>
+      <c r="B22" s="84"/>
       <c r="C22" s="28">
         <f>B21-B22</f>
         <v>0</v>
@@ -2007,13 +1950,13 @@
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="88" t="s">
+      <c r="A27" s="85" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="68"/>
-      <c r="C27" s="68"/>
-      <c r="D27" s="68"/>
-      <c r="E27" s="89">
+      <c r="B27" s="67"/>
+      <c r="C27" s="67"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="86">
         <f>+C27-D27</f>
         <v>0</v>
       </c>
@@ -2024,13 +1967,13 @@
       <c r="G27" s="4"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="88" t="s">
+      <c r="A28" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="B28" s="68"/>
-      <c r="C28" s="68"/>
-      <c r="D28" s="68"/>
-      <c r="E28" s="89"/>
+      <c r="B28" s="67"/>
+      <c r="C28" s="67"/>
+      <c r="D28" s="67"/>
+      <c r="E28" s="86"/>
       <c r="F28" s="41" t="e">
         <f t="shared" ref="F28:F58" si="0">+C28/D28-1</f>
         <v>#DIV/0!</v>
@@ -2038,46 +1981,46 @@
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="67" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" s="69"/>
-      <c r="C29" s="69"/>
-      <c r="D29" s="68"/>
-      <c r="E29" s="90">
+      <c r="A29" s="66" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="68"/>
+      <c r="C29" s="68"/>
+      <c r="D29" s="67"/>
+      <c r="E29" s="87">
         <f>+C29-D29</f>
         <v>0</v>
       </c>
-      <c r="F29" s="65" t="e">
+      <c r="F29" s="64" t="e">
         <f>+C29/D29-1</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G29" s="3"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="77"/>
-      <c r="B30" s="78"/>
-      <c r="C30" s="78"/>
-      <c r="D30" s="68"/>
-      <c r="E30" s="78"/>
-      <c r="F30" s="78"/>
-      <c r="G30" s="64"/>
+      <c r="A30" s="75"/>
+      <c r="B30" s="99"/>
+      <c r="C30" s="99"/>
+      <c r="D30" s="67"/>
+      <c r="E30" s="99"/>
+      <c r="F30" s="76"/>
+      <c r="G30" s="63"/>
       <c r="H30" s="10"/>
       <c r="I30" s="10"/>
       <c r="J30" s="11"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="91" t="s">
+      <c r="A31" s="88" t="s">
         <v>37</v>
       </c>
-      <c r="B31" s="70"/>
-      <c r="C31" s="70"/>
-      <c r="D31" s="68"/>
-      <c r="E31" s="92">
+      <c r="B31" s="69"/>
+      <c r="C31" s="69"/>
+      <c r="D31" s="67"/>
+      <c r="E31" s="89">
         <f>+C31-D31</f>
         <v>0</v>
       </c>
-      <c r="F31" s="66" t="e">
+      <c r="F31" s="65" t="e">
         <f>+C31/D31-1</f>
         <v>#DIV/0!</v>
       </c>
@@ -2087,17 +2030,17 @@
       <c r="J31" s="11"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="67" t="s">
+      <c r="A32" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="69"/>
-      <c r="C32" s="69"/>
-      <c r="D32" s="68"/>
-      <c r="E32" s="90">
+      <c r="B32" s="68"/>
+      <c r="C32" s="68"/>
+      <c r="D32" s="67"/>
+      <c r="E32" s="87">
         <f>+C32-D32</f>
         <v>0</v>
       </c>
-      <c r="F32" s="65" t="e">
+      <c r="F32" s="64" t="e">
         <f>+C32/D32-1</f>
         <v>#DIV/0!</v>
       </c>
@@ -2106,53 +2049,55 @@
       <c r="I32" s="10"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="81"/>
-      <c r="B33" s="79"/>
-      <c r="C33" s="79"/>
-      <c r="D33" s="68"/>
-      <c r="E33" s="79"/>
-      <c r="F33" s="80"/>
-      <c r="G33" s="64"/>
+      <c r="A33" s="79"/>
+      <c r="B33" s="100"/>
+      <c r="C33" s="100"/>
+      <c r="D33" s="67"/>
+      <c r="E33" s="100"/>
+      <c r="F33" s="78"/>
+      <c r="G33" s="63"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="81"/>
-      <c r="B34" s="79"/>
-      <c r="C34" s="79"/>
-      <c r="D34" s="68"/>
-      <c r="E34" s="79"/>
-      <c r="F34" s="80"/>
-      <c r="G34" s="64"/>
+      <c r="A34" s="79"/>
+      <c r="B34" s="100"/>
+      <c r="C34" s="100"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="100"/>
+      <c r="F34" s="78"/>
+      <c r="G34" s="63"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="81"/>
-      <c r="B35" s="79"/>
-      <c r="C35" s="79"/>
-      <c r="D35" s="68"/>
-      <c r="E35" s="79"/>
-      <c r="F35" s="80"/>
-      <c r="G35" s="64"/>
+      <c r="A35" s="79"/>
+      <c r="B35" s="100"/>
+      <c r="C35" s="100"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="100"/>
+      <c r="F35" s="78"/>
+      <c r="G35" s="63"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="77"/>
-      <c r="B36" s="78"/>
-      <c r="C36" s="78"/>
-      <c r="D36" s="68"/>
-      <c r="E36" s="79"/>
-      <c r="F36" s="80"/>
-      <c r="G36" s="64"/>
+      <c r="A36" s="75"/>
+      <c r="B36" s="99"/>
+      <c r="C36" s="99"/>
+      <c r="D36" s="67"/>
+      <c r="E36" s="100"/>
+      <c r="F36" s="78"/>
+      <c r="G36" s="63"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="75" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="72"/>
-      <c r="C37" s="72"/>
-      <c r="D37" s="68"/>
-      <c r="E37" s="93">
+      <c r="B37" s="71">
+        <v>0</v>
+      </c>
+      <c r="C37" s="71"/>
+      <c r="D37" s="67"/>
+      <c r="E37" s="90">
         <f>+C37-D37</f>
         <v>0</v>
       </c>
-      <c r="F37" s="73" t="e">
+      <c r="F37" s="72" t="e">
         <f>+C37/D37-1</f>
         <v>#DIV/0!</v>
       </c>
@@ -2160,239 +2105,229 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="75" t="s">
-        <v>42</v>
-      </c>
-      <c r="B38" s="79"/>
-      <c r="C38" s="79"/>
-      <c r="D38" s="68"/>
-      <c r="E38" s="79"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="64"/>
+        <v>52</v>
+      </c>
+      <c r="B38" s="100"/>
+      <c r="C38" s="100"/>
+      <c r="D38" s="67"/>
+      <c r="E38" s="100">
+        <f t="shared" ref="E38:E41" si="1">+C38-D38</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="78" t="e">
+        <f t="shared" ref="F38:F40" si="2">+C38/D38-1</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G38" s="63"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="75" t="s">
-        <v>52</v>
-      </c>
-      <c r="B39" s="79"/>
-      <c r="C39" s="79"/>
-      <c r="D39" s="68"/>
-      <c r="E39" s="79"/>
-      <c r="F39" s="80"/>
-      <c r="G39" s="64"/>
+      <c r="A39" s="79" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="100"/>
+      <c r="C39" s="100"/>
+      <c r="D39" s="67"/>
+      <c r="E39" s="100">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F39" s="72" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G39" s="63"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="75" t="s">
-        <v>53</v>
-      </c>
-      <c r="B40" s="79"/>
-      <c r="C40" s="79"/>
-      <c r="D40" s="68"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="64"/>
-    </row>
-    <row r="41" spans="1:7" ht="13" x14ac:dyDescent="0.3">
-      <c r="A41" s="75" t="s">
+      <c r="A40" s="79" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="100"/>
+      <c r="C40" s="100"/>
+      <c r="D40" s="67"/>
+      <c r="E40" s="100">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F40" s="77" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G40" s="63"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G41" s="5"/>
+    </row>
+    <row r="42" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A42" s="79"/>
+      <c r="B42" s="101"/>
+      <c r="C42" s="101"/>
+      <c r="D42" s="67"/>
+      <c r="E42" s="100"/>
+      <c r="F42" s="78"/>
+      <c r="G42" s="63"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="75"/>
+      <c r="B43" s="100"/>
+      <c r="C43" s="100"/>
+      <c r="D43" s="67"/>
+      <c r="E43" s="99"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="63"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="74"/>
-      <c r="C41" s="74"/>
-      <c r="D41" s="68"/>
-      <c r="E41" s="93">
-        <f>+C41-D41</f>
-        <v>0</v>
-      </c>
-      <c r="F41" s="73" t="e">
-        <f>+C41/D41-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G41" s="5"/>
-    </row>
-    <row r="42" spans="1:7" ht="13" x14ac:dyDescent="0.3">
-      <c r="A42" s="81"/>
-      <c r="B42" s="82"/>
-      <c r="C42" s="82"/>
-      <c r="D42" s="68"/>
-      <c r="E42" s="79"/>
-      <c r="F42" s="80"/>
-      <c r="G42" s="64"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="77"/>
-      <c r="B43" s="79"/>
-      <c r="C43" s="79"/>
-      <c r="D43" s="68"/>
-      <c r="E43" s="78"/>
-      <c r="F43" s="78"/>
-      <c r="G43" s="64"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="75" t="s">
-        <v>41</v>
-      </c>
-      <c r="B44" s="72"/>
-      <c r="C44" s="72"/>
-      <c r="D44" s="68"/>
-      <c r="E44" s="93">
+      <c r="B44" s="71"/>
+      <c r="C44" s="71"/>
+      <c r="D44" s="67"/>
+      <c r="E44" s="90">
         <f>+C44-D44</f>
         <v>0</v>
       </c>
-      <c r="F44" s="73" t="e">
+      <c r="F44" s="72" t="e">
         <f>+C44/D44-1</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G44" s="5"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="81"/>
-      <c r="B45" s="79"/>
-      <c r="C45" s="79"/>
-      <c r="D45" s="68"/>
-      <c r="E45" s="79"/>
-      <c r="F45" s="80"/>
-      <c r="G45" s="64"/>
+      <c r="A45" s="79"/>
+      <c r="B45" s="100"/>
+      <c r="C45" s="100"/>
+      <c r="D45" s="67"/>
+      <c r="E45" s="100"/>
+      <c r="F45" s="78"/>
+      <c r="G45" s="63"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="81"/>
-      <c r="B46" s="79"/>
-      <c r="C46" s="79"/>
-      <c r="D46" s="68"/>
-      <c r="E46" s="79"/>
-      <c r="F46" s="80"/>
-      <c r="G46" s="64"/>
+      <c r="A46" s="79"/>
+      <c r="B46" s="100"/>
+      <c r="C46" s="100"/>
+      <c r="D46" s="67"/>
+      <c r="E46" s="100"/>
+      <c r="F46" s="78"/>
+      <c r="G46" s="63"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="81"/>
-      <c r="B47" s="79"/>
-      <c r="C47" s="79"/>
-      <c r="D47" s="68"/>
-      <c r="E47" s="79"/>
-      <c r="F47" s="80"/>
-      <c r="G47" s="64"/>
+      <c r="A47" s="79"/>
+      <c r="B47" s="100"/>
+      <c r="C47" s="100"/>
+      <c r="D47" s="67"/>
+      <c r="E47" s="100"/>
+      <c r="F47" s="78"/>
+      <c r="G47" s="63"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="81"/>
-      <c r="B48" s="79"/>
-      <c r="C48" s="79"/>
-      <c r="D48" s="68"/>
-      <c r="E48" s="79"/>
-      <c r="F48" s="80"/>
-      <c r="G48" s="64"/>
+      <c r="A48" s="79"/>
+      <c r="B48" s="100"/>
+      <c r="C48" s="100"/>
+      <c r="D48" s="67"/>
+      <c r="E48" s="100"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="63"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="77"/>
-      <c r="B49" s="78"/>
-      <c r="C49" s="78"/>
-      <c r="D49" s="68"/>
-      <c r="E49" s="78"/>
-      <c r="F49" s="78"/>
-      <c r="G49" s="64"/>
+      <c r="A49" s="75"/>
+      <c r="B49" s="99"/>
+      <c r="C49" s="99"/>
+      <c r="D49" s="67"/>
+      <c r="E49" s="99"/>
+      <c r="F49" s="76"/>
+      <c r="G49" s="63"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="75" t="s">
+      <c r="G50" s="5"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="79"/>
+      <c r="B51" s="77"/>
+      <c r="C51" s="77"/>
+      <c r="D51" s="77"/>
+      <c r="E51" s="77"/>
+      <c r="F51" s="78"/>
+      <c r="G51" s="63"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="79"/>
+      <c r="B52" s="77"/>
+      <c r="C52" s="77"/>
+      <c r="D52" s="77"/>
+      <c r="E52" s="77"/>
+      <c r="F52" s="78"/>
+      <c r="G52" s="63"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="79"/>
+      <c r="B53" s="77"/>
+      <c r="C53" s="77"/>
+      <c r="D53" s="77"/>
+      <c r="E53" s="77"/>
+      <c r="F53" s="78"/>
+      <c r="G53" s="63"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="79"/>
+      <c r="B54" s="77"/>
+      <c r="C54" s="77"/>
+      <c r="D54" s="77"/>
+      <c r="E54" s="77"/>
+      <c r="F54" s="78"/>
+      <c r="G54" s="63"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="79"/>
+      <c r="B55" s="77"/>
+      <c r="C55" s="77"/>
+      <c r="D55" s="77"/>
+      <c r="E55" s="77"/>
+      <c r="F55" s="78"/>
+      <c r="G55" s="63"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="79"/>
+      <c r="B56" s="77"/>
+      <c r="C56" s="77"/>
+      <c r="D56" s="76"/>
+      <c r="E56" s="76"/>
+      <c r="F56" s="76"/>
+      <c r="G56" s="63"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="80"/>
+      <c r="B57" s="77"/>
+      <c r="C57" s="77"/>
+      <c r="D57" s="77"/>
+      <c r="E57" s="77"/>
+      <c r="F57" s="78"/>
+      <c r="G57" s="12"/>
+    </row>
+    <row r="58" spans="1:7" ht="13" x14ac:dyDescent="0.3">
+      <c r="A58" s="74" t="s">
         <v>42</v>
       </c>
-      <c r="B50" s="72"/>
-      <c r="C50" s="72"/>
-      <c r="D50" s="68"/>
-      <c r="E50" s="93">
-        <f>+C50-D50</f>
-        <v>0</v>
-      </c>
-      <c r="F50" s="73" t="e">
-        <f>+C50/D50-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G50" s="5"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="81"/>
-      <c r="B51" s="79"/>
-      <c r="C51" s="79"/>
-      <c r="D51" s="79"/>
-      <c r="E51" s="79"/>
-      <c r="F51" s="80"/>
-      <c r="G51" s="64"/>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="81"/>
-      <c r="B52" s="79"/>
-      <c r="C52" s="79"/>
-      <c r="D52" s="79"/>
-      <c r="E52" s="79"/>
-      <c r="F52" s="80"/>
-      <c r="G52" s="64"/>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="81"/>
-      <c r="B53" s="79"/>
-      <c r="C53" s="79"/>
-      <c r="D53" s="79"/>
-      <c r="E53" s="79"/>
-      <c r="F53" s="80"/>
-      <c r="G53" s="64"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="81"/>
-      <c r="B54" s="79"/>
-      <c r="C54" s="79"/>
-      <c r="D54" s="79"/>
-      <c r="E54" s="79"/>
-      <c r="F54" s="80"/>
-      <c r="G54" s="64"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="81"/>
-      <c r="B55" s="79"/>
-      <c r="C55" s="79"/>
-      <c r="D55" s="79"/>
-      <c r="E55" s="79"/>
-      <c r="F55" s="80"/>
-      <c r="G55" s="64"/>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="81"/>
-      <c r="B56" s="79"/>
-      <c r="C56" s="79"/>
-      <c r="D56" s="78"/>
-      <c r="E56" s="78"/>
-      <c r="F56" s="78"/>
-      <c r="G56" s="64"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="83"/>
-      <c r="B57" s="79"/>
-      <c r="C57" s="79"/>
-      <c r="D57" s="79"/>
-      <c r="E57" s="79"/>
-      <c r="F57" s="80"/>
-      <c r="G57" s="12"/>
-    </row>
-    <row r="58" spans="1:7" ht="13" x14ac:dyDescent="0.3">
-      <c r="A58" s="76" t="s">
-        <v>43</v>
-      </c>
-      <c r="B58" s="71">
+      <c r="B58" s="70">
         <f>SUM(B27:B57)</f>
         <v>0</v>
       </c>
-      <c r="C58" s="71">
-        <f t="shared" ref="C58:D58" si="1">SUM(C27:C57)</f>
+      <c r="C58" s="70">
+        <f t="shared" ref="C58:D58" si="3">SUM(C27:C57)</f>
         <v>0</v>
       </c>
-      <c r="D58" s="71">
-        <f t="shared" si="1"/>
+      <c r="D58" s="70">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="E58" s="92">
-        <f t="shared" ref="E58" si="2">+C58-D58</f>
+      <c r="E58" s="89">
+        <f t="shared" ref="E58" si="4">+C58-D58</f>
         <v>0</v>
       </c>
-      <c r="F58" s="66" t="e">
+      <c r="F58" s="65" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="G58" s="94"/>
+      <c r="G58" s="91"/>
     </row>
     <row r="59" spans="1:7" ht="13" x14ac:dyDescent="0.3">
       <c r="A59" s="7"/>
@@ -2434,12 +2369,12 @@
       <formula>DAY(INDIRECT("$B"&amp;ROW()))=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B27:C29 E27:F29 D27:D50 B31:C35 E41:F42 E44:F48 B50:F55 B56:C56 B57:D57 E57:F58">
+  <conditionalFormatting sqref="B27:C29 E27:F29 D27:D40 B31:C35 E44:F48 B51:F55 B56:C56 B57:D57 E57:F58 D42:D49">
     <cfRule type="cellIs" dxfId="4" priority="6" stopIfTrue="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E31:F39 B37:C48">
+  <conditionalFormatting sqref="E31:F40 B37:C40 B42:C48 E42:F42">
     <cfRule type="cellIs" dxfId="3" priority="2" stopIfTrue="1" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -2449,12 +2384,12 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F27:F29 F31:F39 F41:F42 F44:F48 F50:F55 F57:F58">
+  <conditionalFormatting sqref="F27:F29 F31:F39 F42 F44:F48 F51:F55 F57:F58">
     <cfRule type="cellIs" dxfId="1" priority="17" stopIfTrue="1" operator="lessThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F27:F29 F41:F42 F44:F48 F50:F55 F57:F58 F31:F39">
+  <conditionalFormatting sqref="F27:F29 F44:F48 F51:F55 F57:F58 F31:F39 F42">
     <cfRule type="cellIs" dxfId="0" priority="14" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
@@ -2485,30 +2420,30 @@
   <sheetData>
     <row r="2" spans="2:2" ht="13" x14ac:dyDescent="0.25">
       <c r="B2" s="20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="92" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="2:2" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="95" t="s">
+    <row r="4" spans="2:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="92" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="2:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="95" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="21"/>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B6" s="95" t="s">
-        <v>47</v>
+      <c r="B6" s="92" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="2:2" ht="25" x14ac:dyDescent="0.25">
       <c r="B7" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -2518,26 +2453,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="94dc4dc2-2ec2-43e9-8f94-f5870e81c4cd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ee3cf40a-f169-48b1-a7bd-addeb317f7df" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010053FC4ADBF0C00F469B9370EE17EC2365" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e4926921d97bacc1a28d65a28a31a583">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="94dc4dc2-2ec2-43e9-8f94-f5870e81c4cd" xmlns:ns3="ee3cf40a-f169-48b1-a7bd-addeb317f7df" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dc0f7928e132ab5227fb31a751618f95" ns2:_="" ns3:_="">
     <xsd:import namespace="94dc4dc2-2ec2-43e9-8f94-f5870e81c4cd"/>
@@ -2738,32 +2653,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF7EDB78-65CD-4F80-886F-1A64648DD0AE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A645010A-63C6-47D7-A671-ACFF8009621F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="94dc4dc2-2ec2-43e9-8f94-f5870e81c4cd"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="ee3cf40a-f169-48b1-a7bd-addeb317f7df"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="94dc4dc2-2ec2-43e9-8f94-f5870e81c4cd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ee3cf40a-f169-48b1-a7bd-addeb317f7df" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4575EF5C-54D6-43F7-A522-A72ED8A2CBBB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2780,4 +2690,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF7EDB78-65CD-4F80-886F-1A64648DD0AE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A645010A-63C6-47D7-A671-ACFF8009621F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="94dc4dc2-2ec2-43e9-8f94-f5870e81c4cd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ee3cf40a-f169-48b1-a7bd-addeb317f7df"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>